<commit_message>
adjustemnts to documentation EU5
</commit_message>
<xml_diff>
--- a/docs/games/eu5/calculations & checks.xlsx
+++ b/docs/games/eu5/calculations & checks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PH\Documents\Claude\Projects\PDX Save Analyzer\docs\games\eu5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{10A1141D-5435-45E1-9AB8-579C1E10BAD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79D672FE-8162-4ED8-BDDA-3FCF35A0BF3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{5B610615-9AC8-49E7-8C75-DE8648DC1BA9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="183">
   <si>
     <t>Field</t>
   </si>
@@ -766,7 +766,37 @@
     <t>0.476 (47.6%)</t>
   </si>
   <si>
-    <t>In game found as "wealth of the subjects". 20% of this is used to calculated the "economic base" of the country, alongside</t>
+    <t>no need</t>
+  </si>
+  <si>
+    <t>correct, no need</t>
+  </si>
+  <si>
+    <t>20% of this is used to calculated the "economic base" of the country, alongside population</t>
+  </si>
+  <si>
+    <t>interesting to keep.</t>
+  </si>
+  <si>
+    <t>correct, good to keep</t>
+  </si>
+  <si>
+    <t>don’t know what these are, not displayed in game</t>
+  </si>
+  <si>
+    <t>In game found as "wealth of the subjects". Actually their tax base. So it checks with variable name.</t>
+  </si>
+  <si>
+    <t>missing interests paid (2,22 in current month) and buildings subsidies (currently 0,23) and cost of the court (currently 0)</t>
+  </si>
+  <si>
+    <t>missing court slider</t>
+  </si>
+  <si>
+    <t>missing food sold (+3,62)</t>
+  </si>
+  <si>
+    <t>missing food bought from market (-10,47)</t>
   </si>
 </sst>
 </file>
@@ -815,7 +845,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -837,6 +867,7 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1183,6 +1214,7 @@
     <col min="7" max="7" width="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -1726,6 +1758,9 @@
       <c r="I22" s="1" t="s">
         <v>74</v>
       </c>
+      <c r="J22" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="23" spans="1:15">
       <c r="A23" s="3">
@@ -1753,6 +1788,9 @@
       <c r="I23" s="1" t="s">
         <v>74</v>
       </c>
+      <c r="J23" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="24" spans="1:15">
       <c r="A24" s="3">
@@ -1780,15 +1818,18 @@
       <c r="I24" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="L24">
-        <v>6190</v>
+      <c r="J24" t="s">
+        <v>173</v>
+      </c>
+      <c r="L24" s="11">
+        <v>6190000</v>
       </c>
       <c r="M24">
         <v>92.85</v>
       </c>
       <c r="N24">
         <f>+L24/M24</f>
-        <v>66.666666666666671</v>
+        <v>66666.666666666672</v>
       </c>
       <c r="O24">
         <f>+L24/N24</f>
@@ -1821,6 +1862,9 @@
       <c r="I25" s="1" t="s">
         <v>74</v>
       </c>
+      <c r="J25" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="26" spans="1:15">
       <c r="A26" s="3">
@@ -1848,6 +1892,9 @@
       <c r="I26" s="1" t="s">
         <v>74</v>
       </c>
+      <c r="J26" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="27" spans="1:15">
       <c r="A27" s="3">
@@ -1879,7 +1926,10 @@
         <v>74</v>
       </c>
       <c r="J27" t="s">
-        <v>172</v>
+        <v>178</v>
+      </c>
+      <c r="M27" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="28" spans="1:15">
@@ -1908,6 +1958,9 @@
       <c r="I28" s="1" t="s">
         <v>74</v>
       </c>
+      <c r="J28" t="s">
+        <v>175</v>
+      </c>
     </row>
     <row r="29" spans="1:15">
       <c r="A29" s="3">
@@ -1935,6 +1988,9 @@
       <c r="I29" s="1" t="s">
         <v>74</v>
       </c>
+      <c r="J29" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="30" spans="1:15">
       <c r="A30" s="3">
@@ -1962,11 +2018,21 @@
       <c r="I30" s="1" t="s">
         <v>74</v>
       </c>
+      <c r="J30" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="31" spans="1:15">
       <c r="F31" s="2"/>
-      <c r="G31" s="1"/>
-      <c r="I31" s="1"/>
+      <c r="G31" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J31" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="32" spans="1:15">
       <c r="A32" s="8" t="s">
@@ -1980,7 +2046,7 @@
       <c r="G32" s="1"/>
       <c r="I32" s="1"/>
     </row>
-    <row r="33" spans="1:9">
+    <row r="33" spans="1:10">
       <c r="A33" s="9"/>
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
@@ -1990,7 +2056,7 @@
       <c r="G33" s="1"/>
       <c r="I33" s="1"/>
     </row>
-    <row r="34" spans="1:9">
+    <row r="34" spans="1:10">
       <c r="A34" s="1" t="s">
         <v>76</v>
       </c>
@@ -2006,18 +2072,23 @@
       <c r="E34" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="F34" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Raw Field</v>
+      <c r="F34" s="1" t="s">
+        <v>0</v>
       </c>
       <c r="G34" s="1" t="s">
         <v>74</v>
       </c>
+      <c r="H34" s="1" t="s">
+        <v>66</v>
+      </c>
       <c r="I34" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="35" spans="1:9">
+      <c r="J34" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10">
       <c r="A35" s="3">
         <v>41</v>
       </c>
@@ -2043,8 +2114,11 @@
       <c r="I35" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="36" spans="1:9">
+      <c r="J35" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10">
       <c r="A36" s="3">
         <v>42</v>
       </c>
@@ -2070,8 +2144,11 @@
       <c r="I36" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="37" spans="1:9">
+      <c r="J36" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10">
       <c r="A37" s="3">
         <v>43</v>
       </c>
@@ -2097,8 +2174,11 @@
       <c r="I37" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="38" spans="1:9">
+      <c r="J37" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10">
       <c r="A38" s="3">
         <v>44</v>
       </c>
@@ -2124,8 +2204,11 @@
       <c r="I38" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="39" spans="1:9">
+      <c r="J38" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10">
       <c r="A39" s="3">
         <v>45</v>
       </c>
@@ -2151,8 +2234,11 @@
       <c r="I39" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="40" spans="1:9">
+      <c r="J39" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10">
       <c r="A40" s="3">
         <v>46</v>
       </c>
@@ -2178,8 +2264,11 @@
       <c r="I40" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="41" spans="1:9">
+      <c r="J40" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10">
       <c r="A41" s="3">
         <v>47</v>
       </c>
@@ -2205,8 +2294,11 @@
       <c r="I41" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="42" spans="1:9">
+      <c r="J41" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10">
       <c r="A42" s="3" t="s">
         <v>132</v>
       </c>
@@ -2232,13 +2324,23 @@
       <c r="I42" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="43" spans="1:9">
+      <c r="J42" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10">
       <c r="F43" s="2"/>
-      <c r="G43" s="1"/>
-      <c r="I43" s="1"/>
-    </row>
-    <row r="44" spans="1:9">
+      <c r="G43" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J43" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10">
       <c r="A44" s="8" t="s">
         <v>136</v>
       </c>
@@ -2249,7 +2351,7 @@
       <c r="G44" s="1"/>
       <c r="I44" s="1"/>
     </row>
-    <row r="45" spans="1:9">
+    <row r="45" spans="1:10">
       <c r="A45" s="9"/>
       <c r="B45" s="9"/>
       <c r="C45" s="9"/>
@@ -2258,7 +2360,7 @@
       <c r="G45" s="1"/>
       <c r="I45" s="1"/>
     </row>
-    <row r="46" spans="1:9">
+    <row r="46" spans="1:10">
       <c r="A46" s="1" t="s">
         <v>76</v>
       </c>
@@ -2271,18 +2373,23 @@
       <c r="D46" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="F46" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Raw Field</v>
+      <c r="F46" s="1" t="s">
+        <v>0</v>
       </c>
       <c r="G46" s="1" t="s">
         <v>74</v>
       </c>
+      <c r="H46" s="1" t="s">
+        <v>66</v>
+      </c>
       <c r="I46" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="47" spans="1:9">
+      <c r="J46" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10">
       <c r="A47" s="3">
         <v>48</v>
       </c>
@@ -2306,7 +2413,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="48" spans="1:9">
+    <row r="48" spans="1:10">
       <c r="A48" s="3">
         <v>49</v>
       </c>
@@ -2330,7 +2437,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="49" spans="1:9">
+    <row r="49" spans="1:10">
       <c r="A49" s="3">
         <v>50</v>
       </c>
@@ -2353,8 +2460,11 @@
       <c r="I49" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="50" spans="1:9">
+      <c r="J49" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10">
       <c r="A50" s="3">
         <v>51</v>
       </c>
@@ -2377,8 +2487,11 @@
       <c r="I50" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="51" spans="1:9">
+      <c r="J50" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10">
       <c r="A51" s="9"/>
       <c r="B51" s="9"/>
       <c r="C51" s="9"/>
@@ -2387,7 +2500,7 @@
       <c r="G51" s="1"/>
       <c r="I51" s="1"/>
     </row>
-    <row r="52" spans="1:9">
+    <row r="52" spans="1:10">
       <c r="A52" s="8" t="s">
         <v>149</v>
       </c>
@@ -2398,7 +2511,7 @@
       <c r="G52" s="1"/>
       <c r="I52" s="1"/>
     </row>
-    <row r="53" spans="1:9">
+    <row r="53" spans="1:10">
       <c r="A53" s="9"/>
       <c r="B53" s="9"/>
       <c r="C53" s="9"/>
@@ -2407,7 +2520,7 @@
       <c r="G53" s="1"/>
       <c r="I53" s="1"/>
     </row>
-    <row r="54" spans="1:9">
+    <row r="54" spans="1:10">
       <c r="A54" s="1" t="s">
         <v>150</v>
       </c>
@@ -2418,9 +2531,20 @@
         <v>152</v>
       </c>
       <c r="D54" s="9"/>
-      <c r="F54" s="2"/>
-    </row>
-    <row r="55" spans="1:9">
+      <c r="F54" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="I54" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10">
       <c r="A55" s="3" t="s">
         <v>153</v>
       </c>
@@ -2431,9 +2555,23 @@
         <v>155</v>
       </c>
       <c r="D55" s="9"/>
-      <c r="F55" s="2"/>
-    </row>
-    <row r="56" spans="1:9">
+      <c r="F55" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H55" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="I55" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J55" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10">
       <c r="A56" s="3" t="s">
         <v>156</v>
       </c>
@@ -2444,9 +2582,23 @@
         <v>1</v>
       </c>
       <c r="D56" s="9"/>
-      <c r="F56" s="2"/>
-    </row>
-    <row r="57" spans="1:9">
+      <c r="F56" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="I56" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J56" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10">
       <c r="A57" s="3" t="s">
         <v>157</v>
       </c>
@@ -2457,9 +2609,23 @@
         <v>1</v>
       </c>
       <c r="D57" s="9"/>
-      <c r="F57" s="2"/>
-    </row>
-    <row r="58" spans="1:9">
+      <c r="F57" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H57" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="I57" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J57" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10">
       <c r="A58" s="3" t="s">
         <v>158</v>
       </c>
@@ -2470,9 +2636,23 @@
         <v>0.25</v>
       </c>
       <c r="D58" s="9"/>
-      <c r="F58" s="2"/>
-    </row>
-    <row r="59" spans="1:9">
+      <c r="F58" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="I58" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J58" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10">
       <c r="A59" s="3" t="s">
         <v>160</v>
       </c>
@@ -2483,9 +2663,23 @@
         <v>0.5</v>
       </c>
       <c r="D59" s="9"/>
-      <c r="F59" s="2"/>
-    </row>
-    <row r="60" spans="1:9">
+      <c r="F59" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H59" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="I59" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J59" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10">
       <c r="A60" s="3" t="s">
         <v>162</v>
       </c>
@@ -2496,32 +2690,59 @@
         <v>0.5</v>
       </c>
       <c r="D60" s="9"/>
-      <c r="F60" s="2"/>
-    </row>
-    <row r="61" spans="1:9">
+      <c r="F60" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H60" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="I60" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J60" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10">
       <c r="A61" s="9"/>
       <c r="B61" s="9"/>
       <c r="C61" s="9"/>
       <c r="D61" s="9"/>
       <c r="F61" s="2"/>
-    </row>
-    <row r="62" spans="1:9">
+      <c r="G61" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="I61" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J61" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10">
       <c r="A62" s="8" t="s">
         <v>163</v>
       </c>
       <c r="B62" s="9"/>
       <c r="C62" s="9"/>
       <c r="D62" s="9"/>
-      <c r="F62" s="2"/>
-    </row>
-    <row r="63" spans="1:9">
+      <c r="F62" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="H62" s="9"/>
+    </row>
+    <row r="63" spans="1:10">
       <c r="A63" s="9"/>
       <c r="B63" s="9"/>
       <c r="C63" s="9"/>
       <c r="D63" s="9"/>
-      <c r="F63" s="2"/>
-    </row>
-    <row r="64" spans="1:9">
+      <c r="F63" s="9"/>
+      <c r="H63" s="9"/>
+    </row>
+    <row r="64" spans="1:10">
       <c r="A64" s="1" t="s">
         <v>164</v>
       </c>
@@ -2530,9 +2751,20 @@
       </c>
       <c r="C64" s="9"/>
       <c r="D64" s="9"/>
-      <c r="F64" s="2"/>
-    </row>
-    <row r="65" spans="1:6">
+      <c r="F64" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="G64" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H64" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="I64" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10">
       <c r="A65" s="3" t="s">
         <v>166</v>
       </c>
@@ -2541,9 +2773,23 @@
       </c>
       <c r="C65" s="9"/>
       <c r="D65" s="9"/>
-      <c r="F65" s="2"/>
-    </row>
-    <row r="66" spans="1:6">
+      <c r="F65" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H65" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="I65" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J65" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10">
       <c r="A66" s="3" t="s">
         <v>168</v>
       </c>
@@ -2552,9 +2798,23 @@
       </c>
       <c r="C66" s="9"/>
       <c r="D66" s="9"/>
-      <c r="F66" s="2"/>
-    </row>
-    <row r="67" spans="1:6">
+      <c r="F66" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H66" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="I66" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J66" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10">
       <c r="A67" s="3" t="s">
         <v>170</v>
       </c>
@@ -2563,9 +2823,23 @@
       </c>
       <c r="C67" s="9"/>
       <c r="D67" s="9"/>
-      <c r="F67" s="2"/>
-    </row>
-    <row r="68" spans="1:6">
+      <c r="F67" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J67" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10">
       <c r="F68" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
documentation refinement- diplo, religio, wars
</commit_message>
<xml_diff>
--- a/docs/games/eu5/calculations & checks.xlsx
+++ b/docs/games/eu5/calculations & checks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PH\Documents\Claude\Projects\PDX Save Analyzer\docs\games\eu5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79D672FE-8162-4ED8-BDDA-3FCF35A0BF3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E7580BC-56D6-4391-9549-E656B33F655B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{5B610615-9AC8-49E7-8C75-DE8648DC1BA9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="268">
   <si>
     <t>Field</t>
   </si>
@@ -797,6 +797,291 @@
   </si>
   <si>
     <t>missing food bought from market (-10,47)</t>
+  </si>
+  <si>
+    <t>Counter</t>
+  </si>
+  <si>
+    <t>FRA value</t>
+  </si>
+  <si>
+    <t>Proposed meaning</t>
+  </si>
+  <si>
+    <t>Track?</t>
+  </si>
+  <si>
+    <t>Advances</t>
+  </si>
+  <si>
+    <t>Total advances researched</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>Anything</t>
+  </si>
+  <si>
+    <t>Total events fired? Global event count?</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>BorderLocations</t>
+  </si>
+  <si>
+    <t>Number of border locations</t>
+  </si>
+  <si>
+    <t>BuildingLevelChanged</t>
+  </si>
+  <si>
+    <t>Total building level changes over game</t>
+  </si>
+  <si>
+    <t>CabinetCardModifier</t>
+  </si>
+  <si>
+    <t>Cabinet card interactions?</t>
+  </si>
+  <si>
+    <t>CoastalLocations</t>
+  </si>
+  <si>
+    <t>Coastal locations owned</t>
+  </si>
+  <si>
+    <t>ConstructionStarted</t>
+  </si>
+  <si>
+    <t>Total constructions ever started</t>
+  </si>
+  <si>
+    <t>Diplomacy</t>
+  </si>
+  <si>
+    <t>Total diplomatic actions taken</t>
+  </si>
+  <si>
+    <t>DiscoveredLocations</t>
+  </si>
+  <si>
+    <t>Locations explored/discovered</t>
+  </si>
+  <si>
+    <t>LivingCharacters</t>
+  </si>
+  <si>
+    <t>Current living characters associated</t>
+  </si>
+  <si>
+    <t>Locations</t>
+  </si>
+  <si>
+    <t>Total locations owned</t>
+  </si>
+  <si>
+    <t>Pops</t>
+  </si>
+  <si>
+    <t>Total pops</t>
+  </si>
+  <si>
+    <r>
+      <t>YES</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (vs </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>last_months_population</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>PrimaryCulture</t>
+  </si>
+  <si>
+    <t>Times primary culture changed</t>
+  </si>
+  <si>
+    <t>RGO</t>
+  </si>
+  <si>
+    <t>RGO (resource gathering operations) count</t>
+  </si>
+  <si>
+    <t>Rebels</t>
+  </si>
+  <si>
+    <t>Total rebel events?</t>
+  </si>
+  <si>
+    <t>Reforms</t>
+  </si>
+  <si>
+    <t>Government reforms enacted</t>
+  </si>
+  <si>
+    <t>Siege</t>
+  </si>
+  <si>
+    <t>Total sieges</t>
+  </si>
+  <si>
+    <t>SubjectTree</t>
+  </si>
+  <si>
+    <t>Subject/vassal nodes</t>
+  </si>
+  <si>
+    <t>TradePath</t>
+  </si>
+  <si>
+    <t>Trade paths</t>
+  </si>
+  <si>
+    <t>Wars</t>
+  </si>
+  <si>
+    <t>Total wars participated in</t>
+  </si>
+  <si>
+    <t>WorksOfArt</t>
+  </si>
+  <si>
+    <t>Works of art created</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>str</t>
+  </si>
+  <si>
+    <t>'nobles'</t>
+  </si>
+  <si>
+    <t>estate</t>
+  </si>
+  <si>
+    <t>'nobles_estate'</t>
+  </si>
+  <si>
+    <t>culture</t>
+  </si>
+  <si>
+    <t>int</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>'Primary'</t>
+  </si>
+  <si>
+    <t>religion</t>
+  </si>
+  <si>
+    <t>satisfaction</t>
+  </si>
+  <si>
+    <t>float</t>
+  </si>
+  <si>
+    <t>0.5892</t>
+  </si>
+  <si>
+    <t>size</t>
+  </si>
+  <si>
+    <t>0.224</t>
+  </si>
+  <si>
+    <t>literacy</t>
+  </si>
+  <si>
+    <t>goods</t>
+  </si>
+  <si>
+    <t>0.9259</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>-0.05307</t>
+  </si>
+  <si>
+    <t>missing</t>
+  </si>
+  <si>
+    <t>dict</t>
+  </si>
+  <si>
+    <t>(3 keys)</t>
+  </si>
+  <si>
+    <t>NOT really: the "pops" are entities identified by an ID (115951 keys in population database), carrying a size component (for example pop #0 has a size of 0,224); locations list every pop belonging there; these locations are then assigned to a owner country. So the sum of the size of each pops of each location of a country would be the total population.</t>
+  </si>
+  <si>
+    <t>Total pops objects in population node</t>
+  </si>
+  <si>
+    <t>every country has 2 here, so let's simply ignore</t>
+  </si>
+  <si>
+    <t>RGO Level count</t>
+  </si>
+  <si>
+    <t>Total rebel movements/groups ever created</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>No but document as investigation topic</t>
+  </si>
+  <si>
+    <t>no idea, skip</t>
+  </si>
+  <si>
+    <t>Commented meaning</t>
+  </si>
+  <si>
+    <t>other notes:</t>
+  </si>
+  <si>
+    <t>the UI shows 70 advances researched, your number might be off here. Before we go any further please let me know what is the country ID of France and the current in game date?</t>
+  </si>
+  <si>
+    <t>researched_advances</t>
+  </si>
+  <si>
+    <t>the count should suffice for now</t>
   </si>
 </sst>
 </file>
@@ -845,7 +1130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -862,12 +1147,11 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -883,6 +1167,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>29288</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>114646</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2704529E-DC96-80C6-1DF3-94BBC7E456AA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="20564475" y="9067800"/>
+          <a:ext cx="5106113" cy="2476846"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1202,10 +1535,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFD1EA9A-9546-452A-AB26-F904639CEB2A}">
-  <dimension ref="A1:O68"/>
+  <dimension ref="A1:T94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="45.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="37.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="35.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.140625" bestFit="1" customWidth="1"/>
@@ -1213,8 +1546,10 @@
     <col min="6" max="6" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="46.140625" customWidth="1"/>
+    <col min="11" max="11" width="2.28515625" customWidth="1"/>
     <col min="12" max="12" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -1685,20 +2020,9 @@
       </c>
     </row>
     <row r="19" spans="1:15">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-    </row>
-    <row r="20" spans="1:15">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
     </row>
     <row r="21" spans="1:15">
       <c r="A21" s="1" t="s">
@@ -1779,7 +2103,7 @@
         <v>86</v>
       </c>
       <c r="F23" s="2" t="str">
-        <f t="shared" ref="F23:F68" si="0">B23</f>
+        <f t="shared" ref="F23:F50" si="0">B23</f>
         <v>estimated_monthly_income</v>
       </c>
       <c r="G23" s="1" t="s">
@@ -1821,7 +2145,7 @@
       <c r="J24" t="s">
         <v>173</v>
       </c>
-      <c r="L24" s="11">
+      <c r="L24" s="9">
         <v>6190000</v>
       </c>
       <c r="M24">
@@ -2035,23 +2359,14 @@
       </c>
     </row>
     <row r="32" spans="1:15">
-      <c r="A32" s="8" t="s">
+      <c r="A32" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="B32" s="9"/>
-      <c r="C32" s="9"/>
-      <c r="D32" s="9"/>
-      <c r="E32" s="9"/>
       <c r="F32" s="2"/>
       <c r="G32" s="1"/>
       <c r="I32" s="1"/>
     </row>
     <row r="33" spans="1:10">
-      <c r="A33" s="9"/>
-      <c r="B33" s="9"/>
-      <c r="C33" s="9"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="9"/>
       <c r="F33" s="2"/>
       <c r="G33" s="1"/>
       <c r="I33" s="1"/>
@@ -2341,21 +2656,14 @@
       </c>
     </row>
     <row r="44" spans="1:10">
-      <c r="A44" s="8" t="s">
+      <c r="A44" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="B44" s="9"/>
-      <c r="C44" s="9"/>
-      <c r="D44" s="9"/>
       <c r="F44" s="2"/>
       <c r="G44" s="1"/>
       <c r="I44" s="1"/>
     </row>
     <row r="45" spans="1:10">
-      <c r="A45" s="9"/>
-      <c r="B45" s="9"/>
-      <c r="C45" s="9"/>
-      <c r="D45" s="9"/>
       <c r="F45" s="2"/>
       <c r="G45" s="1"/>
       <c r="I45" s="1"/>
@@ -2492,30 +2800,19 @@
       </c>
     </row>
     <row r="51" spans="1:10">
-      <c r="A51" s="9"/>
-      <c r="B51" s="9"/>
-      <c r="C51" s="9"/>
-      <c r="D51" s="9"/>
       <c r="F51" s="2"/>
       <c r="G51" s="1"/>
       <c r="I51" s="1"/>
     </row>
     <row r="52" spans="1:10">
-      <c r="A52" s="8" t="s">
+      <c r="A52" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="B52" s="9"/>
-      <c r="C52" s="9"/>
-      <c r="D52" s="9"/>
       <c r="F52" s="2"/>
       <c r="G52" s="1"/>
       <c r="I52" s="1"/>
     </row>
     <row r="53" spans="1:10">
-      <c r="A53" s="9"/>
-      <c r="B53" s="9"/>
-      <c r="C53" s="9"/>
-      <c r="D53" s="9"/>
       <c r="F53" s="2"/>
       <c r="G53" s="1"/>
       <c r="I53" s="1"/>
@@ -2530,7 +2827,6 @@
       <c r="C54" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="D54" s="9"/>
       <c r="F54" s="1" t="s">
         <v>150</v>
       </c>
@@ -2554,7 +2850,6 @@
       <c r="C55" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="D55" s="9"/>
       <c r="F55" s="3" t="s">
         <v>153</v>
       </c>
@@ -2578,10 +2873,9 @@
       <c r="B56" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="C56" s="10">
+      <c r="C56" s="8">
         <v>1</v>
       </c>
-      <c r="D56" s="9"/>
       <c r="F56" s="3" t="s">
         <v>156</v>
       </c>
@@ -2605,10 +2899,9 @@
       <c r="B57" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="C57" s="10">
+      <c r="C57" s="8">
         <v>1</v>
       </c>
-      <c r="D57" s="9"/>
       <c r="F57" s="3" t="s">
         <v>157</v>
       </c>
@@ -2632,10 +2925,9 @@
       <c r="B58" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="C58" s="10">
+      <c r="C58" s="8">
         <v>0.25</v>
       </c>
-      <c r="D58" s="9"/>
       <c r="F58" s="3" t="s">
         <v>158</v>
       </c>
@@ -2659,10 +2951,9 @@
       <c r="B59" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="C59" s="10">
+      <c r="C59" s="8">
         <v>0.5</v>
       </c>
-      <c r="D59" s="9"/>
       <c r="F59" s="3" t="s">
         <v>160</v>
       </c>
@@ -2686,10 +2977,9 @@
       <c r="B60" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="C60" s="10">
+      <c r="C60" s="8">
         <v>0.5</v>
       </c>
-      <c r="D60" s="9"/>
       <c r="F60" s="3" t="s">
         <v>162</v>
       </c>
@@ -2707,10 +2997,6 @@
       </c>
     </row>
     <row r="61" spans="1:10">
-      <c r="A61" s="9"/>
-      <c r="B61" s="9"/>
-      <c r="C61" s="9"/>
-      <c r="D61" s="9"/>
       <c r="F61" s="2"/>
       <c r="G61" s="1" t="s">
         <v>74</v>
@@ -2723,24 +3009,12 @@
       </c>
     </row>
     <row r="62" spans="1:10">
-      <c r="A62" s="8" t="s">
+      <c r="A62" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="B62" s="9"/>
-      <c r="C62" s="9"/>
-      <c r="D62" s="9"/>
-      <c r="F62" s="8" t="s">
+      <c r="F62" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="H62" s="9"/>
-    </row>
-    <row r="63" spans="1:10">
-      <c r="A63" s="9"/>
-      <c r="B63" s="9"/>
-      <c r="C63" s="9"/>
-      <c r="D63" s="9"/>
-      <c r="F63" s="9"/>
-      <c r="H63" s="9"/>
     </row>
     <row r="64" spans="1:10">
       <c r="A64" s="1" t="s">
@@ -2749,8 +3023,6 @@
       <c r="B64" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="C64" s="9"/>
-      <c r="D64" s="9"/>
       <c r="F64" s="1" t="s">
         <v>164</v>
       </c>
@@ -2764,15 +3036,13 @@
         <v>74</v>
       </c>
     </row>
-    <row r="65" spans="1:10">
+    <row r="65" spans="1:20">
       <c r="A65" s="3" t="s">
         <v>166</v>
       </c>
       <c r="B65" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="C65" s="9"/>
-      <c r="D65" s="9"/>
       <c r="F65" s="3" t="s">
         <v>166</v>
       </c>
@@ -2789,15 +3059,13 @@
         <v>176</v>
       </c>
     </row>
-    <row r="66" spans="1:10">
+    <row r="66" spans="1:20">
       <c r="A66" s="3" t="s">
         <v>168</v>
       </c>
       <c r="B66" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="C66" s="9"/>
-      <c r="D66" s="9"/>
       <c r="F66" s="3" t="s">
         <v>168</v>
       </c>
@@ -2813,16 +3081,23 @@
       <c r="J66" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="67" spans="1:10">
+      <c r="R66" t="s">
+        <v>232</v>
+      </c>
+      <c r="S66" t="s">
+        <v>233</v>
+      </c>
+      <c r="T66" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="67" spans="1:20">
       <c r="A67" s="3" t="s">
         <v>170</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C67" s="9"/>
-      <c r="D67" s="9"/>
       <c r="F67" s="3" t="s">
         <v>170</v>
       </c>
@@ -2838,11 +3113,807 @@
       <c r="J67" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="68" spans="1:10">
+      <c r="R67" t="s">
+        <v>235</v>
+      </c>
+      <c r="S67" t="s">
+        <v>233</v>
+      </c>
+      <c r="T67" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="68" spans="1:20">
       <c r="F68" s="2"/>
+      <c r="R68" t="s">
+        <v>237</v>
+      </c>
+      <c r="S68" t="s">
+        <v>238</v>
+      </c>
+      <c r="T68">
+        <v>1846</v>
+      </c>
+    </row>
+    <row r="69" spans="1:20" s="10" customFormat="1">
+      <c r="A69" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="G69" s="1"/>
+      <c r="H69" s="1"/>
+      <c r="I69" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J69" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="K69" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L69" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="R69" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="S69" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="T69" s="10" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="70" spans="1:20" s="10" customFormat="1">
+      <c r="A70" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B70" s="3">
+        <v>177</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="D70" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="G70" s="1"/>
+      <c r="H70" s="3"/>
+      <c r="I70" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J70" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="K70" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L70" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="R70" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="S70" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="T70" s="10">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="71" spans="1:20" s="10" customFormat="1">
+      <c r="A71" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B71" s="3">
+        <v>12.961</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="G71" s="1"/>
+      <c r="H71" s="3"/>
+      <c r="I71" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J71" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K71" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L71" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="R71" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="S71" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="T71" s="10" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="72" spans="1:20" s="10" customFormat="1">
+      <c r="A72" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B72" s="3">
+        <v>177</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="D72" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="G72" s="1"/>
+      <c r="H72" s="3"/>
+      <c r="I72" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J72" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="K72" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L72" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="R72" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="S72" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="T72" s="10" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="73" spans="1:20" s="10" customFormat="1">
+      <c r="A73" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B73" s="3">
+        <v>1.46</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="D73" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="G73" s="1"/>
+      <c r="H73" s="3"/>
+      <c r="I73" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J73" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="K73" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L73" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="R73" s="10" t="s">
+        <v>247</v>
+      </c>
+      <c r="S73" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="T73" s="10">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="74" spans="1:20" s="10" customFormat="1">
+      <c r="A74" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B74" s="3">
+        <v>500</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G74" s="1"/>
+      <c r="H74" s="3"/>
+      <c r="I74" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J74" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="K74" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L74" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="R74" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="S74" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="T74" s="10" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="75" spans="1:20" s="10" customFormat="1">
+      <c r="A75" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B75" s="3">
+        <v>64</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G75" s="1"/>
+      <c r="H75" s="3"/>
+      <c r="I75" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J75" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="K75" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L75" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="R75" s="10" t="s">
+        <v>250</v>
+      </c>
+      <c r="S75" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="T75" s="10" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="76" spans="1:20" s="10" customFormat="1">
+      <c r="A76" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B76" s="3">
+        <v>1.1419999999999999</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="G76" s="1"/>
+      <c r="H76" s="3"/>
+      <c r="I76" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J76" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="K76" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L76" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="R76" s="10" t="s">
+        <v>252</v>
+      </c>
+      <c r="S76" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="T76" s="10" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="77" spans="1:20" s="10" customFormat="1">
+      <c r="A77" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B77" s="3">
+        <v>3.59</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="G77" s="1"/>
+      <c r="H77" s="3"/>
+      <c r="I77" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J77" s="3" t="str">
+        <f>C77</f>
+        <v>Total diplomatic actions taken</v>
+      </c>
+      <c r="K77" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L77" s="3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="78" spans="1:20" s="10" customFormat="1">
+      <c r="A78" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B78" s="3">
+        <v>329</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="D78" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="G78" s="1"/>
+      <c r="H78" s="3"/>
+      <c r="I78" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J78" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="K78" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L78" s="5" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="79" spans="1:20" s="10" customFormat="1">
+      <c r="A79" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B79" s="3">
+        <v>1.486</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="G79" s="1"/>
+      <c r="H79" s="3"/>
+      <c r="I79" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J79" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="K79" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L79" s="3" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="80" spans="1:20" s="10" customFormat="1">
+      <c r="A80" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B80" s="3">
+        <v>339</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="D80" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="G80" s="1"/>
+      <c r="H80" s="3"/>
+      <c r="I80" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J80" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="K80" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L80" s="5" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" s="10" customFormat="1">
+      <c r="A81" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B81" s="3">
+        <v>1.7569999999999999</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="D81" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="G81" s="1"/>
+      <c r="H81" s="3"/>
+      <c r="I81" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J81" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="K81" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L81" s="5" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" s="10" customFormat="1">
+      <c r="A82" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B82" s="3">
+        <v>2</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="G82" s="1"/>
+      <c r="H82" s="3"/>
+      <c r="I82" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J82" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="K82" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L82" s="3" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" s="10" customFormat="1">
+      <c r="A83" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B83" s="3">
+        <v>1.018</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="D83" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="F83" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="G83" s="1"/>
+      <c r="H83" s="3"/>
+      <c r="I83" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J83" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="K83" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L83" s="5" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" s="10" customFormat="1">
+      <c r="A84" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B84" s="3">
+        <v>122</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="G84" s="1"/>
+      <c r="H84" s="3"/>
+      <c r="I84" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J84" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="K84" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L84" s="3" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" s="10" customFormat="1">
+      <c r="A85" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B85" s="3">
+        <v>3</v>
+      </c>
+      <c r="C85" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="D85" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="G85" s="1"/>
+      <c r="H85" s="3"/>
+      <c r="I85" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J85" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="K85" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L85" s="5" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" s="10" customFormat="1">
+      <c r="A86" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B86" s="3">
+        <v>83</v>
+      </c>
+      <c r="C86" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="G86" s="1"/>
+      <c r="H86" s="3"/>
+      <c r="I86" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J86" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="K86" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L86" s="3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" s="10" customFormat="1">
+      <c r="A87" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B87" s="3">
+        <v>104</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D87" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="G87" s="1"/>
+      <c r="H87" s="3"/>
+      <c r="I87" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J87" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="K87" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L87" s="3" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" s="10" customFormat="1">
+      <c r="A88" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B88" s="3">
+        <v>329</v>
+      </c>
+      <c r="C88" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="D88" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F88" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="G88" s="1"/>
+      <c r="H88" s="3"/>
+      <c r="I88" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J88" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="K88" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L88" s="3" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" s="10" customFormat="1">
+      <c r="A89" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B89" s="3">
+        <v>295</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D89" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="F89" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="G89" s="1"/>
+      <c r="H89" s="3"/>
+      <c r="I89" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J89" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="K89" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L89" s="5" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" s="10" customFormat="1">
+      <c r="A90" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B90" s="3">
+        <v>3</v>
+      </c>
+      <c r="C90" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F90" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="G90" s="1"/>
+      <c r="H90" s="3"/>
+      <c r="I90" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J90" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="K90" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L90" s="3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12">
+      <c r="F92" s="2" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12">
+      <c r="F93" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="J93" s="3" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12">
+      <c r="F94" t="s">
+        <v>266</v>
+      </c>
+      <c r="J94" s="3" t="s">
+        <v>267</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>